<commit_message>
Update: Stable Build v0.2
</commit_message>
<xml_diff>
--- a/APPT/data/input/latest_uploaded_data.xlsx
+++ b/APPT/data/input/latest_uploaded_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="199">
   <si>
     <t>Production Line</t>
   </si>
@@ -58,126 +58,135 @@
     <t>INT3</t>
   </si>
   <si>
-    <t>910731092</t>
-  </si>
-  <si>
-    <t>910730950</t>
-  </si>
-  <si>
-    <t>910731190</t>
-  </si>
-  <si>
-    <t>910731146</t>
-  </si>
-  <si>
-    <t>910730970</t>
-  </si>
-  <si>
-    <t>910731173</t>
-  </si>
-  <si>
-    <t>910731091</t>
-  </si>
-  <si>
-    <t>910730951</t>
-  </si>
-  <si>
-    <t>910731192</t>
-  </si>
-  <si>
-    <t>910731148</t>
-  </si>
-  <si>
-    <t>910730972</t>
-  </si>
-  <si>
-    <t>910730971</t>
-  </si>
-  <si>
-    <t>910731147</t>
-  </si>
-  <si>
-    <t>910731172</t>
-  </si>
-  <si>
-    <t>910731189</t>
-  </si>
-  <si>
-    <t>910731090</t>
-  </si>
-  <si>
-    <t>910731145</t>
-  </si>
-  <si>
-    <t>910730969</t>
-  </si>
-  <si>
-    <t>910731062</t>
-  </si>
-  <si>
-    <t>910731115</t>
-  </si>
-  <si>
-    <t>910731102</t>
-  </si>
-  <si>
-    <t>910730963</t>
-  </si>
-  <si>
-    <t>910730943</t>
-  </si>
-  <si>
-    <t>910731125</t>
-  </si>
-  <si>
-    <t>910731168</t>
-  </si>
-  <si>
-    <t>910731183</t>
-  </si>
-  <si>
-    <t>910731220</t>
-  </si>
-  <si>
-    <t>910731319</t>
-  </si>
-  <si>
-    <t>910731238</t>
-  </si>
-  <si>
-    <t>910731304</t>
-  </si>
-  <si>
-    <t>910731210</t>
-  </si>
-  <si>
-    <t>910731292</t>
-  </si>
-  <si>
-    <t>910731221</t>
-  </si>
-  <si>
-    <t>910731293</t>
-  </si>
-  <si>
-    <t>910728784</t>
-  </si>
-  <si>
-    <t>910728850</t>
-  </si>
-  <si>
-    <t>910731057</t>
-  </si>
-  <si>
-    <t>910730961</t>
-  </si>
-  <si>
-    <t>910731031</t>
+    <t>910720379</t>
+  </si>
+  <si>
+    <t>910720583</t>
+  </si>
+  <si>
+    <t>910722008</t>
+  </si>
+  <si>
+    <t>910722037</t>
+  </si>
+  <si>
+    <t>910722009</t>
+  </si>
+  <si>
+    <t>910721917</t>
+  </si>
+  <si>
+    <t>910721947</t>
+  </si>
+  <si>
+    <t>910721945</t>
+  </si>
+  <si>
+    <t>910721946</t>
+  </si>
+  <si>
+    <t>910721918</t>
+  </si>
+  <si>
+    <t>910720351</t>
+  </si>
+  <si>
+    <t>910720600</t>
+  </si>
+  <si>
+    <t>910722016</t>
+  </si>
+  <si>
+    <t>910722007</t>
+  </si>
+  <si>
+    <t>910722035</t>
+  </si>
+  <si>
+    <t>910722006</t>
+  </si>
+  <si>
+    <t>910721981</t>
+  </si>
+  <si>
+    <t>910722018</t>
+  </si>
+  <si>
+    <t>910721944</t>
+  </si>
+  <si>
+    <t>910721919</t>
+  </si>
+  <si>
+    <t>910720484</t>
+  </si>
+  <si>
+    <t>910720547</t>
+  </si>
+  <si>
+    <t>910720590</t>
+  </si>
+  <si>
+    <t>910720486</t>
+  </si>
+  <si>
+    <t>910720524</t>
+  </si>
+  <si>
+    <t>910723317</t>
+  </si>
+  <si>
+    <t>910722156</t>
+  </si>
+  <si>
+    <t>910722206</t>
+  </si>
+  <si>
+    <t>910722089</t>
+  </si>
+  <si>
+    <t>910722128</t>
+  </si>
+  <si>
+    <t>910723069</t>
+  </si>
+  <si>
+    <t>910722903</t>
+  </si>
+  <si>
+    <t>910723000</t>
+  </si>
+  <si>
+    <t>910717129</t>
+  </si>
+  <si>
+    <t>910717198</t>
+  </si>
+  <si>
+    <t>910722166</t>
+  </si>
+  <si>
+    <t>910722371</t>
+  </si>
+  <si>
+    <t>910722385</t>
+  </si>
+  <si>
+    <t>910722300</t>
+  </si>
+  <si>
+    <t>910722223</t>
   </si>
   <si>
     <t>83900263</t>
   </si>
   <si>
+    <t>83900258</t>
+  </si>
+  <si>
+    <t>83900206</t>
+  </si>
+  <si>
     <t>83900261</t>
   </si>
   <si>
@@ -187,63 +196,60 @@
     <t>83900259</t>
   </si>
   <si>
-    <t>83900260</t>
+    <t>80879287</t>
+  </si>
+  <si>
+    <t>80879283</t>
+  </si>
+  <si>
+    <t>80879271</t>
+  </si>
+  <si>
+    <t>80879274</t>
+  </si>
+  <si>
+    <t>80880911</t>
   </si>
   <si>
     <t>80880893</t>
   </si>
   <si>
-    <t>80880901</t>
-  </si>
-  <si>
-    <t>80880900</t>
+    <t>80880890</t>
+  </si>
+  <si>
+    <t>80880895</t>
+  </si>
+  <si>
+    <t>80879273</t>
   </si>
   <si>
     <t>80880914</t>
   </si>
   <si>
-    <t>80880904</t>
-  </si>
-  <si>
-    <t>80879274</t>
-  </si>
-  <si>
-    <t>80879275</t>
-  </si>
-  <si>
-    <t>80879288</t>
-  </si>
-  <si>
-    <t>80879278</t>
-  </si>
-  <si>
-    <t>80879287</t>
-  </si>
-  <si>
-    <t>80879283</t>
-  </si>
-  <si>
-    <t>80880910</t>
-  </si>
-  <si>
-    <t>80880916</t>
-  </si>
-  <si>
-    <t>80841061</t>
+    <t>80896958</t>
+  </si>
+  <si>
+    <t>80830098</t>
+  </si>
+  <si>
+    <t>80878378</t>
   </si>
   <si>
     <t>80841060</t>
   </si>
   <si>
-    <t>80851522</t>
-  </si>
-  <si>
-    <t>80878378</t>
+    <t>80851521</t>
   </si>
   <si>
     <t>H&amp;S SHM 5.7MLX960 DAILY CLEAN IN GST FC</t>
   </si>
   <si>
+    <t>H&amp;S SHM 5.7MLX1200 NEEM IN GST FC</t>
+  </si>
+  <si>
+    <t>H&amp;S SHM 5.7MLX960 NEEM IN GST FC</t>
+  </si>
+  <si>
     <t>H&amp;S SHM 5.7MLX 960 DS IN GST FC</t>
   </si>
   <si>
@@ -253,310 +259,319 @@
     <t>H&amp;S SHM 5.7MLX1200 DAILY CLEAN IN GST FC</t>
   </si>
   <si>
-    <t>H&amp;S SHM 5.7MLX960 DAILY COOL IN GST FC</t>
+    <t>PNTN SHM 650ML X 12 HFC GST</t>
+  </si>
+  <si>
+    <t>PNTN SHM 650ML X 12 SSC IN GST</t>
+  </si>
+  <si>
+    <t>PNTN SHM 340ML X 30 HS SS IN GST</t>
+  </si>
+  <si>
+    <t>PNTN SHM 340MLX30 HS HFC IN GST</t>
+  </si>
+  <si>
+    <t>H&amp;S SHM 180ML X 56 CM 2IN1 IN GST</t>
   </si>
   <si>
     <t>H&amp;S SHM 180ML X 56 AHF IN GST</t>
   </si>
   <si>
-    <t>H&amp;S SHM 180ML X 56 LF IN GST</t>
-  </si>
-  <si>
-    <t>H&amp;S SHM 300ML X30 CM IN DM GST</t>
+    <t>H&amp;S SHM 180ML X 56 SB IN GST</t>
+  </si>
+  <si>
+    <t>H&amp;S SHM 180ML X 56 CM IN GST</t>
+  </si>
+  <si>
+    <t>PNTN SHM 75 MLX48 HS HFC IN GST</t>
   </si>
   <si>
     <t>H&amp;S SHM 340ML X30 CM IN GST</t>
   </si>
   <si>
-    <t>H&amp;S SHM 340ML X30 AHF IN GST</t>
-  </si>
-  <si>
-    <t>PNTN SHM 340MLX30 HS HFC IN GST</t>
-  </si>
-  <si>
-    <t>PNTN SHM 340ML X 30 HS LT IN GST</t>
-  </si>
-  <si>
-    <t>PNTN SHM 180ML X 56 HS LT IN GST</t>
-  </si>
-  <si>
-    <t>PNTN SHM 180MLX56 HS HFC IN GST</t>
-  </si>
-  <si>
-    <t>PNTN SHM 650ML X 12 HFC GST</t>
-  </si>
-  <si>
-    <t>PNTN SHM 650ML X 12 SSC IN GST</t>
-  </si>
-  <si>
-    <t>H&amp;S SHM 650ML X12 AHF IN GST</t>
-  </si>
-  <si>
-    <t>H&amp;S SHM 650ML X12 CM IN GST</t>
-  </si>
-  <si>
-    <t>PNTN COND 200MLX 24 HS HF IN PC25</t>
+    <t>H&amp;S SHM 340ML X 30 S&amp;S IN GST Promo 7in1</t>
+  </si>
+  <si>
+    <t>PNTN 3MM BIOTIN COND 200MLX24 IN</t>
+  </si>
+  <si>
+    <t>PNTN 3MM COLLAGEN CONDI 80MLX24 IN GST</t>
   </si>
   <si>
     <t>PNTN COND 200MLX 24 HS SS IN PC25</t>
   </si>
   <si>
-    <t>PNTN COND 100MLX 24 HS HF IN AMJ25</t>
-  </si>
-  <si>
-    <t>PNTN 3MM COLLAGEN CONDI 80MLX24 IN GST</t>
-  </si>
-  <si>
-    <t>6015930219</t>
-  </si>
-  <si>
-    <t>6015930214</t>
-  </si>
-  <si>
-    <t>6015930216</t>
-  </si>
-  <si>
-    <t>6015930217</t>
-  </si>
-  <si>
-    <t>6016930211</t>
-  </si>
-  <si>
-    <t>6016930212</t>
-  </si>
-  <si>
-    <t>6016930213</t>
-  </si>
-  <si>
-    <t>6016930214</t>
-  </si>
-  <si>
-    <t>6016930215</t>
-  </si>
-  <si>
-    <t>601593024B</t>
-  </si>
-  <si>
-    <t>601593024C</t>
-  </si>
-  <si>
-    <t>6015930249</t>
-  </si>
-  <si>
-    <t>6015930248</t>
-  </si>
-  <si>
-    <t>6015930247</t>
-  </si>
-  <si>
-    <t>6016930247</t>
-  </si>
-  <si>
-    <t>6016930248</t>
-  </si>
-  <si>
-    <t>6016930249</t>
-  </si>
-  <si>
-    <t>6016930246</t>
-  </si>
-  <si>
-    <t>6015930264</t>
-  </si>
-  <si>
-    <t>6015930263</t>
-  </si>
-  <si>
-    <t>6015930266</t>
-  </si>
-  <si>
-    <t>6015930265</t>
-  </si>
-  <si>
-    <t>6015930268</t>
-  </si>
-  <si>
-    <t>6015930267</t>
-  </si>
-  <si>
-    <t>601593026A</t>
-  </si>
-  <si>
-    <t>6015930269</t>
-  </si>
-  <si>
-    <t>601593026B</t>
-  </si>
-  <si>
-    <t>6016930265</t>
-  </si>
-  <si>
-    <t>6016930263</t>
-  </si>
-  <si>
-    <t>6016930264</t>
-  </si>
-  <si>
-    <t>6016930262</t>
-  </si>
-  <si>
-    <t>6016930261</t>
-  </si>
-  <si>
-    <t>6016930267</t>
-  </si>
-  <si>
-    <t>6016930266</t>
-  </si>
-  <si>
-    <t>6015930281</t>
-  </si>
-  <si>
-    <t>6015930280</t>
-  </si>
-  <si>
-    <t>6016930281</t>
-  </si>
-  <si>
-    <t>6016930280</t>
-  </si>
-  <si>
-    <t>6017930280</t>
-  </si>
-  <si>
-    <t>15.01.2026</t>
-  </si>
-  <si>
-    <t>16.01.2026</t>
-  </si>
-  <si>
-    <t>17.01.2026</t>
-  </si>
-  <si>
-    <t>06:53</t>
-  </si>
-  <si>
-    <t>11:18</t>
-  </si>
-  <si>
-    <t>15:43</t>
-  </si>
-  <si>
-    <t>20:07</t>
-  </si>
-  <si>
-    <t>00:32</t>
-  </si>
-  <si>
-    <t>04:56</t>
-  </si>
-  <si>
-    <t>09:21</t>
-  </si>
-  <si>
-    <t>13:45</t>
-  </si>
-  <si>
-    <t>18:10</t>
-  </si>
-  <si>
-    <t>06:00</t>
-  </si>
-  <si>
-    <t>11:07</t>
-  </si>
-  <si>
-    <t>13:41</t>
+    <t>PNTN COND 100MLX 24 HS SS IN AMJ25</t>
+  </si>
+  <si>
+    <t>6009930216</t>
+  </si>
+  <si>
+    <t>6010930211</t>
+  </si>
+  <si>
+    <t>6010930212</t>
+  </si>
+  <si>
+    <t>6010930213</t>
+  </si>
+  <si>
+    <t>6011930217</t>
+  </si>
+  <si>
+    <t>6011930215</t>
+  </si>
+  <si>
+    <t>6011930218</t>
+  </si>
+  <si>
+    <t>6011930216</t>
+  </si>
+  <si>
+    <t>6012930214</t>
+  </si>
+  <si>
+    <t>6012930215</t>
+  </si>
+  <si>
+    <t>6008930249</t>
+  </si>
+  <si>
+    <t>6010930242</t>
+  </si>
+  <si>
+    <t>6010930243</t>
+  </si>
+  <si>
+    <t>601193024A</t>
+  </si>
+  <si>
+    <t>6011930249</t>
+  </si>
+  <si>
+    <t>6011930246</t>
+  </si>
+  <si>
+    <t>6011930247</t>
+  </si>
+  <si>
+    <t>601193024B</t>
+  </si>
+  <si>
+    <t>6011930248</t>
+  </si>
+  <si>
+    <t>601193024C</t>
+  </si>
+  <si>
+    <t>6009930263</t>
+  </si>
+  <si>
+    <t>6010930260</t>
+  </si>
+  <si>
+    <t>6010930262</t>
+  </si>
+  <si>
+    <t>6010930263</t>
+  </si>
+  <si>
+    <t>6010930261</t>
+  </si>
+  <si>
+    <t>6010930268</t>
+  </si>
+  <si>
+    <t>6010930267</t>
+  </si>
+  <si>
+    <t>6010930266</t>
+  </si>
+  <si>
+    <t>6010930264</t>
+  </si>
+  <si>
+    <t>6010930265</t>
+  </si>
+  <si>
+    <t>6011930268</t>
+  </si>
+  <si>
+    <t>6011930266</t>
+  </si>
+  <si>
+    <t>6011930267</t>
+  </si>
+  <si>
+    <t>6008930281</t>
+  </si>
+  <si>
+    <t>6008930280</t>
+  </si>
+  <si>
+    <t>6010930280</t>
+  </si>
+  <si>
+    <t>6010930281</t>
+  </si>
+  <si>
+    <t>6011930280</t>
+  </si>
+  <si>
+    <t>6011930281</t>
+  </si>
+  <si>
+    <t>6012930280</t>
+  </si>
+  <si>
+    <t>09.01.2026</t>
+  </si>
+  <si>
+    <t>10.01.2026</t>
+  </si>
+  <si>
+    <t>11.01.2026</t>
+  </si>
+  <si>
+    <t>12.01.2026</t>
+  </si>
+  <si>
+    <t>08.01.2026</t>
+  </si>
+  <si>
+    <t>06:44</t>
+  </si>
+  <si>
+    <t>11:08</t>
+  </si>
+  <si>
+    <t>15:33</t>
+  </si>
+  <si>
+    <t>19:58</t>
+  </si>
+  <si>
+    <t>08:22</t>
+  </si>
+  <si>
+    <t>12:47</t>
+  </si>
+  <si>
+    <t>17:11</t>
+  </si>
+  <si>
+    <t>21:36</t>
+  </si>
+  <si>
+    <t>02:00</t>
+  </si>
+  <si>
+    <t>06:25</t>
+  </si>
+  <si>
+    <t>22:09</t>
+  </si>
+  <si>
+    <t>08:43</t>
+  </si>
+  <si>
+    <t>13:50</t>
+  </si>
+  <si>
+    <t>00:24</t>
+  </si>
+  <si>
+    <t>02:58</t>
+  </si>
+  <si>
+    <t>05:32</t>
+  </si>
+  <si>
+    <t>08:05</t>
+  </si>
+  <si>
+    <t>13:13</t>
+  </si>
+  <si>
+    <t>18:20</t>
+  </si>
+  <si>
+    <t>23:28</t>
+  </si>
+  <si>
+    <t>06:12</t>
+  </si>
+  <si>
+    <t>09:05</t>
+  </si>
+  <si>
+    <t>10:32</t>
+  </si>
+  <si>
+    <t>11:59</t>
+  </si>
+  <si>
+    <t>14:00</t>
+  </si>
+  <si>
+    <t>14:37</t>
+  </si>
+  <si>
+    <t>16:16</t>
+  </si>
+  <si>
+    <t>18:31</t>
+  </si>
+  <si>
+    <t>20:47</t>
+  </si>
+  <si>
+    <t>23:03</t>
+  </si>
+  <si>
+    <t>13:00</t>
+  </si>
+  <si>
+    <t>13:43</t>
+  </si>
+  <si>
+    <t>14:26</t>
+  </si>
+  <si>
+    <t>10:00</t>
+  </si>
+  <si>
+    <t>14:19</t>
+  </si>
+  <si>
+    <t>10:01</t>
+  </si>
+  <si>
+    <t>13:58</t>
+  </si>
+  <si>
+    <t>10:23</t>
+  </si>
+  <si>
+    <t>10:50</t>
+  </si>
+  <si>
+    <t>04:35</t>
+  </si>
+  <si>
+    <t>13:25</t>
   </si>
   <si>
     <t>16:15</t>
   </si>
   <si>
-    <t>21:22</t>
-  </si>
-  <si>
-    <t>02:30</t>
-  </si>
-  <si>
-    <t>07:37</t>
-  </si>
-  <si>
-    <t>12:44</t>
-  </si>
-  <si>
-    <t>17:52</t>
-  </si>
-  <si>
-    <t>07:30</t>
-  </si>
-  <si>
-    <t>09:45</t>
-  </si>
-  <si>
-    <t>12:01</t>
-  </si>
-  <si>
-    <t>13:24</t>
-  </si>
-  <si>
-    <t>15:18</t>
-  </si>
-  <si>
-    <t>16:45</t>
-  </si>
-  <si>
-    <t>18:12</t>
-  </si>
-  <si>
-    <t>19:38</t>
-  </si>
-  <si>
-    <t>22:31</t>
-  </si>
-  <si>
-    <t>08:00</t>
-  </si>
-  <si>
-    <t>09:08</t>
-  </si>
-  <si>
-    <t>11:23</t>
-  </si>
-  <si>
-    <t>12:50</t>
-  </si>
-  <si>
-    <t>14:17</t>
-  </si>
-  <si>
-    <t>15:44</t>
-  </si>
-  <si>
-    <t>17:10</t>
-  </si>
-  <si>
-    <t>09:51</t>
-  </si>
-  <si>
-    <t>14:10</t>
-  </si>
-  <si>
-    <t>10:13</t>
-  </si>
-  <si>
-    <t>14:31</t>
-  </si>
-  <si>
-    <t>22:35</t>
-  </si>
-  <si>
-    <t>23:00</t>
-  </si>
-  <si>
-    <t>23:15</t>
-  </si>
-  <si>
-    <t>18:37</t>
+    <t>12:20</t>
+  </si>
+  <si>
+    <t>15:53</t>
+  </si>
+  <si>
+    <t>14:20</t>
   </si>
   <si>
     <t>2,076</t>
@@ -565,31 +580,34 @@
     <t>830</t>
   </si>
   <si>
+    <t>1,038</t>
+  </si>
+  <si>
     <t>1,660</t>
   </si>
   <si>
+    <t>1,484</t>
+  </si>
+  <si>
+    <t>742</t>
+  </si>
+  <si>
+    <t>570</t>
+  </si>
+  <si>
+    <t>160</t>
+  </si>
+  <si>
+    <t>415</t>
+  </si>
+  <si>
     <t>575</t>
   </si>
   <si>
-    <t>420</t>
-  </si>
-  <si>
-    <t>750</t>
-  </si>
-  <si>
-    <t>570</t>
-  </si>
-  <si>
-    <t>1,140</t>
+    <t>1,564</t>
   </si>
   <si>
     <t>285</t>
-  </si>
-  <si>
-    <t>288</t>
-  </si>
-  <si>
-    <t>742</t>
   </si>
   <si>
     <t>300</t>
@@ -950,7 +968,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -993,28 +1011,28 @@
         <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D2" t="s">
         <v>75</v>
       </c>
       <c r="E2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F2" t="s">
         <v>136</v>
       </c>
       <c r="G2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="J2" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -1025,28 +1043,28 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D3" t="s">
         <v>75</v>
       </c>
       <c r="E3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="J3" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -1057,28 +1075,28 @@
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D4" t="s">
         <v>75</v>
       </c>
       <c r="E4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G4" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="H4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I4" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="J4" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -1089,28 +1107,28 @@
         <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D5" t="s">
         <v>75</v>
       </c>
       <c r="E5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="H5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="J5" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -1121,28 +1139,28 @@
         <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D6" t="s">
         <v>75</v>
       </c>
       <c r="E6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G6" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="J6" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -1153,28 +1171,28 @@
         <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D7" t="s">
         <v>75</v>
       </c>
       <c r="E7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="H7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I7" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="J7" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -1185,28 +1203,28 @@
         <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D8" t="s">
         <v>75</v>
       </c>
       <c r="E8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G8" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I8" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="J8" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -1217,28 +1235,28 @@
         <v>21</v>
       </c>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D9" t="s">
         <v>75</v>
       </c>
       <c r="E9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F9" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G9" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="H9" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I9" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="J9" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -1249,33 +1267,33 @@
         <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D10" t="s">
         <v>75</v>
       </c>
       <c r="E10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F10" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G10" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="H10" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I10" t="s">
-        <v>177</v>
+        <v>150</v>
       </c>
       <c r="J10" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
         <v>23</v>
@@ -1284,25 +1302,25 @@
         <v>54</v>
       </c>
       <c r="D11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F11" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G11" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H11" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="I11" t="s">
-        <v>149</v>
+        <v>179</v>
       </c>
       <c r="J11" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -1316,25 +1334,25 @@
         <v>55</v>
       </c>
       <c r="D12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F12" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="G12" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H12" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I12" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J12" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -1345,28 +1363,28 @@
         <v>25</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D13" t="s">
         <v>77</v>
       </c>
       <c r="E13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F13" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G13" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H13" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="J13" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -1377,28 +1395,28 @@
         <v>26</v>
       </c>
       <c r="C14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D14" t="s">
         <v>78</v>
       </c>
       <c r="E14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F14" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G14" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="H14" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="I14" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="J14" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -1409,28 +1427,28 @@
         <v>27</v>
       </c>
       <c r="C15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D15" t="s">
         <v>78</v>
       </c>
       <c r="E15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F15" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G15" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H15" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I15" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="J15" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -1441,28 +1459,28 @@
         <v>28</v>
       </c>
       <c r="C16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D16" t="s">
         <v>78</v>
       </c>
       <c r="E16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F16" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G16" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H16" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I16" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="J16" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -1473,28 +1491,28 @@
         <v>29</v>
       </c>
       <c r="C17" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E17" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F17" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G17" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="H17" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I17" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="J17" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -1505,28 +1523,28 @@
         <v>30</v>
       </c>
       <c r="C18" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E18" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F18" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G18" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H18" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I18" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="J18" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -1537,65 +1555,65 @@
         <v>31</v>
       </c>
       <c r="C19" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D19" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F19" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G19" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H19" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I19" t="s">
-        <v>178</v>
+        <v>159</v>
       </c>
       <c r="J19" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B20" t="s">
         <v>32</v>
       </c>
       <c r="C20" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D20" t="s">
         <v>80</v>
       </c>
       <c r="E20" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F20" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G20" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="H20" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="I20" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="J20" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B21" t="s">
         <v>33</v>
@@ -1604,25 +1622,25 @@
         <v>59</v>
       </c>
       <c r="D21" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E21" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F21" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G21" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H21" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="I21" t="s">
-        <v>159</v>
+        <v>180</v>
       </c>
       <c r="J21" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -1636,25 +1654,25 @@
         <v>60</v>
       </c>
       <c r="D22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E22" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F22" t="s">
         <v>136</v>
       </c>
       <c r="G22" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="H22" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I22" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="J22" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -1668,25 +1686,25 @@
         <v>61</v>
       </c>
       <c r="D23" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E23" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F23" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G23" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H23" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I23" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J23" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -1697,28 +1715,28 @@
         <v>36</v>
       </c>
       <c r="C24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D24" t="s">
         <v>83</v>
       </c>
       <c r="E24" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F24" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G24" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="H24" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I24" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="J24" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -1729,28 +1747,28 @@
         <v>37</v>
       </c>
       <c r="C25" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D25" t="s">
         <v>84</v>
       </c>
       <c r="E25" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F25" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G25" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="H25" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I25" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="J25" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -1761,28 +1779,28 @@
         <v>38</v>
       </c>
       <c r="C26" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D26" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E26" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F26" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G26" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="H26" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I26" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="J26" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -1793,28 +1811,28 @@
         <v>39</v>
       </c>
       <c r="C27" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D27" t="s">
         <v>85</v>
       </c>
       <c r="E27" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F27" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G27" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H27" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I27" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
       <c r="J27" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -1825,28 +1843,28 @@
         <v>40</v>
       </c>
       <c r="C28" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D28" t="s">
         <v>86</v>
       </c>
       <c r="E28" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F28" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G28" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H28" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I28" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="J28" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -1857,28 +1875,28 @@
         <v>41</v>
       </c>
       <c r="C29" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D29" t="s">
         <v>87</v>
       </c>
       <c r="E29" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F29" t="s">
         <v>137</v>
       </c>
       <c r="G29" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H29" t="s">
         <v>137</v>
       </c>
       <c r="I29" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="J29" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -1889,28 +1907,28 @@
         <v>42</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D30" t="s">
         <v>88</v>
       </c>
       <c r="E30" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F30" t="s">
         <v>137</v>
       </c>
       <c r="G30" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="H30" t="s">
         <v>137</v>
       </c>
       <c r="I30" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="J30" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -1921,28 +1939,28 @@
         <v>43</v>
       </c>
       <c r="C31" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D31" t="s">
         <v>89</v>
       </c>
       <c r="E31" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F31" t="s">
         <v>137</v>
       </c>
       <c r="G31" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="H31" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I31" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="J31" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -1953,28 +1971,28 @@
         <v>44</v>
       </c>
       <c r="C32" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D32" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E32" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G32" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="H32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I32" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="J32" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -1985,28 +2003,28 @@
         <v>45</v>
       </c>
       <c r="C33" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D33" t="s">
         <v>90</v>
       </c>
       <c r="E33" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F33" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G33" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="H33" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I33" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="J33" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
     </row>
     <row r="34" spans="1:10">
@@ -2017,60 +2035,60 @@
         <v>46</v>
       </c>
       <c r="C34" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D34" t="s">
         <v>91</v>
       </c>
       <c r="E34" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F34" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G34" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="H34" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I34" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="J34" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B35" t="s">
         <v>47</v>
       </c>
       <c r="C35" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D35" t="s">
         <v>92</v>
       </c>
       <c r="E35" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F35" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="G35" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="H35" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="I35" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="J35" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
     </row>
     <row r="36" spans="1:10">
@@ -2081,28 +2099,28 @@
         <v>48</v>
       </c>
       <c r="C36" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D36" t="s">
         <v>93</v>
       </c>
       <c r="E36" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F36" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="G36" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="H36" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I36" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="J36" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -2113,28 +2131,28 @@
         <v>49</v>
       </c>
       <c r="C37" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D37" t="s">
         <v>93</v>
       </c>
       <c r="E37" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F37" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G37" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="H37" t="s">
         <v>137</v>
       </c>
       <c r="I37" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="J37" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -2145,28 +2163,28 @@
         <v>50</v>
       </c>
       <c r="C38" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D38" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E38" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F38" t="s">
         <v>137</v>
       </c>
       <c r="G38" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H38" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I38" t="s">
         <v>176</v>
       </c>
       <c r="J38" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="39" spans="1:10">
@@ -2180,13 +2198,13 @@
         <v>73</v>
       </c>
       <c r="D39" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E39" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F39" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G39" t="s">
         <v>176</v>
@@ -2198,7 +2216,7 @@
         <v>175</v>
       </c>
       <c r="J39" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="40" spans="1:10">
@@ -2209,13 +2227,13 @@
         <v>52</v>
       </c>
       <c r="C40" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D40" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E40" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F40" t="s">
         <v>138</v>
@@ -2224,13 +2242,45 @@
         <v>175</v>
       </c>
       <c r="H40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I40" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="J40" t="s">
-        <v>192</v>
+        <v>198</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10">
+      <c r="A41" t="s">
+        <v>13</v>
+      </c>
+      <c r="B41" t="s">
+        <v>53</v>
+      </c>
+      <c r="C41" t="s">
+        <v>74</v>
+      </c>
+      <c r="D41" t="s">
+        <v>95</v>
+      </c>
+      <c r="E41" t="s">
+        <v>135</v>
+      </c>
+      <c r="F41" t="s">
+        <v>139</v>
+      </c>
+      <c r="G41" t="s">
+        <v>178</v>
+      </c>
+      <c r="H41" t="s">
+        <v>139</v>
+      </c>
+      <c r="I41" t="s">
+        <v>185</v>
+      </c>
+      <c r="J41" t="s">
+        <v>198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>